<commit_message>
add Pungitius pungitius and Chironomus riparius
</commit_message>
<xml_diff>
--- a/mutation_rate_literature_updating3.xlsx
+++ b/mutation_rate_literature_updating3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yigua\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1F8AF0-0FF8-4FFB-8783-7A13BC10B601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D6E892-3F83-478E-A8F2-50A613BB8FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{09A42BD9-4349-4213-8D0A-A379C870C482}"/>
+    <workbookView xWindow="7800" yWindow="6810" windowWidth="26370" windowHeight="11460" xr2:uid="{09A42BD9-4349-4213-8D0A-A379C870C482}"/>
   </bookViews>
   <sheets>
     <sheet name="raw" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9622" uniqueCount="2673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9686" uniqueCount="2702">
   <si>
     <t>PID</t>
   </si>
@@ -8415,6 +8415,120 @@
   </si>
   <si>
     <t>https://genome.cshlp.org/content/early/2015/05/05/gr185041114</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>fish</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>nine-spined stickleback</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pungitius pungitius</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Baltic Sea (Marine)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Finland and Sweden (fresh water)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>4.63e-9</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.74e-9</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>DNBseq</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>35X</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026006_01</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026006_02</t>
+  </si>
+  <si>
+    <t>https://www.biorxiv.org/content/10.64898/2026.07.31.741990v1</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Chaowei Zhang, Hongbo Wang, Kerry Reid, Dandan Wang, Lei Lv, Yvette Heimbrand, Mikkel Heide Schierup, Juha Merila. (2026). Intra-specific evidence to support the drift-barrier hypothesis of mutation rate evolution. Biorxiv.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>MA</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>30X</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>gatk</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hessen, Germany</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Andalusia, Spain</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>5.71e-9</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.02e-9</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>non-biting midge</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Chironomus riparius</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">arthropods  </t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>arthropods</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026007_01</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026007_02</t>
+  </si>
+  <si>
+    <t>Pfenninger, M., M. E. Nieto-Blazquez, and B. Bulut. 2026. “ Divergent Thermal Reaction Norms of the Spontaneous Mutation Rate Among Populations of Chironomus riparius.” Molecular Ecology 35, no. 15: e70503. https://doi.org/10.1111/mec.70503.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://onlinelibrary.wiley.com/doi/10.1111/mec.70503</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>temperature-dependent</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -8516,7 +8630,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -8535,19 +8649,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -8864,7 +8976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{318201D5-CE15-42FE-AD6F-C948F9B6134A}">
-  <dimension ref="A1:AC556"/>
+  <dimension ref="A1:AC560"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="5.75" customWidth="1"/>
@@ -37619,64 +37731,64 @@
         <v>1691</v>
       </c>
     </row>
-    <row r="429" spans="1:29" s="14" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A429" s="14">
+    <row r="429" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A429">
         <v>2022008</v>
       </c>
-      <c r="B429" s="14">
+      <c r="B429">
         <v>2022</v>
       </c>
-      <c r="C429" s="14" t="s">
+      <c r="C429" t="s">
         <v>37</v>
       </c>
-      <c r="D429" s="14" t="s">
+      <c r="D429" t="s">
         <v>2242</v>
       </c>
-      <c r="E429" s="14" t="s">
+      <c r="E429" t="s">
         <v>214</v>
       </c>
-      <c r="F429" s="14" t="s">
+      <c r="F429" t="s">
         <v>1722</v>
       </c>
-      <c r="H429" s="14" t="s">
+      <c r="H429" t="s">
         <v>1723</v>
       </c>
-      <c r="I429" s="14" t="s">
+      <c r="I429" t="s">
         <v>2013</v>
       </c>
-      <c r="J429" s="14" t="s">
+      <c r="J429" t="s">
         <v>30</v>
       </c>
-      <c r="K429" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="L429" s="15" t="s">
+      <c r="K429" t="s">
+        <v>31</v>
+      </c>
+      <c r="L429" s="4" t="s">
         <v>1724</v>
       </c>
-      <c r="M429" s="15"/>
-      <c r="N429" s="15"/>
-      <c r="O429" s="15"/>
-      <c r="P429" s="15"/>
-      <c r="Q429" s="15"/>
-      <c r="R429" s="15" t="s">
+      <c r="M429" s="4"/>
+      <c r="N429" s="4"/>
+      <c r="O429" s="4"/>
+      <c r="P429" s="4"/>
+      <c r="Q429" s="4"/>
+      <c r="R429" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="S429" s="15"/>
-      <c r="T429" s="15" t="s">
+      <c r="S429" s="4"/>
+      <c r="T429" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="U429" s="15"/>
-      <c r="V429" s="15"/>
-      <c r="W429" s="15" t="s">
+      <c r="U429" s="4"/>
+      <c r="V429" s="4"/>
+      <c r="W429" s="4" t="s">
         <v>1689</v>
       </c>
-      <c r="X429" s="15"/>
-      <c r="Y429" s="15"/>
-      <c r="Z429" s="15"/>
-      <c r="AA429" s="15" t="s">
+      <c r="X429" s="4"/>
+      <c r="Y429" s="4"/>
+      <c r="Z429" s="4"/>
+      <c r="AA429" s="4" t="s">
         <v>1725</v>
       </c>
-      <c r="AC429" s="16" t="s">
+      <c r="AC429" s="14" t="s">
         <v>1726</v>
       </c>
     </row>
@@ -44957,68 +45069,68 @@
         <v>2591</v>
       </c>
     </row>
-    <row r="551" spans="1:29" s="17" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A551" s="17">
+    <row r="551" spans="1:29" s="15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A551" s="15">
         <v>2026001</v>
       </c>
-      <c r="B551" s="17">
+      <c r="B551" s="15">
         <v>2026</v>
       </c>
-      <c r="C551" s="17" t="s">
+      <c r="C551" s="15" t="s">
         <v>2354</v>
       </c>
-      <c r="D551" s="17" t="s">
+      <c r="D551" s="15" t="s">
         <v>2354</v>
       </c>
-      <c r="E551" s="18" t="s">
+      <c r="E551" s="16" t="s">
         <v>2355</v>
       </c>
-      <c r="F551" s="17" t="s">
+      <c r="F551" s="15" t="s">
         <v>2356</v>
       </c>
-      <c r="G551" s="17" t="s">
+      <c r="G551" s="15" t="s">
         <v>2297</v>
       </c>
-      <c r="H551" s="17" t="s">
+      <c r="H551" s="15" t="s">
         <v>2357</v>
       </c>
-      <c r="I551" s="17" t="s">
+      <c r="I551" s="15" t="s">
         <v>2358</v>
       </c>
-      <c r="J551" s="17" t="s">
+      <c r="J551" s="15" t="s">
         <v>2359</v>
       </c>
-      <c r="K551" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="L551" s="19" t="s">
+      <c r="K551" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="L551" s="17" t="s">
         <v>2360</v>
       </c>
-      <c r="M551" s="20" t="s">
+      <c r="M551" s="18" t="s">
         <v>2361</v>
       </c>
-      <c r="N551" s="20" t="s">
+      <c r="N551" s="18" t="s">
         <v>2362</v>
       </c>
-      <c r="R551" s="21">
+      <c r="R551" s="19">
         <v>100</v>
       </c>
-      <c r="S551" s="17">
+      <c r="S551" s="15">
         <v>8765896425</v>
       </c>
-      <c r="T551" s="22" t="s">
+      <c r="T551" s="20" t="s">
         <v>2304</v>
       </c>
-      <c r="U551" s="17">
+      <c r="U551" s="15">
         <v>4</v>
       </c>
-      <c r="Y551" s="17" t="s">
+      <c r="Y551" s="15" t="s">
         <v>2363</v>
       </c>
-      <c r="AA551" s="17" t="s">
+      <c r="AA551" s="15" t="s">
         <v>2364</v>
       </c>
-      <c r="AC551" s="23" t="s">
+      <c r="AC551" s="21" t="s">
         <v>2365</v>
       </c>
     </row>
@@ -45288,6 +45400,254 @@
       </c>
       <c r="AC556" s="1" t="s">
         <v>2490</v>
+      </c>
+    </row>
+    <row r="557" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A557">
+        <v>2026006</v>
+      </c>
+      <c r="B557">
+        <v>2026</v>
+      </c>
+      <c r="C557" t="s">
+        <v>2673</v>
+      </c>
+      <c r="D557" t="s">
+        <v>2673</v>
+      </c>
+      <c r="E557" s="7" t="s">
+        <v>2674</v>
+      </c>
+      <c r="F557" t="s">
+        <v>2675</v>
+      </c>
+      <c r="G557" t="s">
+        <v>2677</v>
+      </c>
+      <c r="H557" t="s">
+        <v>2682</v>
+      </c>
+      <c r="I557" t="s">
+        <v>2299</v>
+      </c>
+      <c r="J557" t="s">
+        <v>2286</v>
+      </c>
+      <c r="K557" t="s">
+        <v>31</v>
+      </c>
+      <c r="L557" s="13" t="s">
+        <v>2678</v>
+      </c>
+      <c r="R557" s="8">
+        <v>472</v>
+      </c>
+      <c r="T557" s="4" t="s">
+        <v>2304</v>
+      </c>
+      <c r="U557">
+        <v>164</v>
+      </c>
+      <c r="W557" s="4" t="s">
+        <v>2680</v>
+      </c>
+      <c r="Y557" t="s">
+        <v>2681</v>
+      </c>
+      <c r="AA557" t="s">
+        <v>2685</v>
+      </c>
+      <c r="AC557" s="1" t="s">
+        <v>2684</v>
+      </c>
+    </row>
+    <row r="558" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A558">
+        <v>2026006</v>
+      </c>
+      <c r="B558">
+        <v>2026</v>
+      </c>
+      <c r="C558" t="s">
+        <v>2673</v>
+      </c>
+      <c r="D558" t="s">
+        <v>2673</v>
+      </c>
+      <c r="E558" s="7" t="s">
+        <v>2674</v>
+      </c>
+      <c r="F558" t="s">
+        <v>2675</v>
+      </c>
+      <c r="G558" t="s">
+        <v>2676</v>
+      </c>
+      <c r="H558" t="s">
+        <v>2683</v>
+      </c>
+      <c r="I558" t="s">
+        <v>2299</v>
+      </c>
+      <c r="J558" t="s">
+        <v>2286</v>
+      </c>
+      <c r="K558" t="s">
+        <v>31</v>
+      </c>
+      <c r="L558" s="13" t="s">
+        <v>2679</v>
+      </c>
+      <c r="R558" s="8">
+        <v>463</v>
+      </c>
+      <c r="T558" s="4" t="s">
+        <v>2304</v>
+      </c>
+      <c r="U558">
+        <v>218</v>
+      </c>
+      <c r="W558" s="4" t="s">
+        <v>2680</v>
+      </c>
+      <c r="Y558" t="s">
+        <v>2681</v>
+      </c>
+      <c r="AA558" t="s">
+        <v>2685</v>
+      </c>
+      <c r="AC558" s="1" t="s">
+        <v>2684</v>
+      </c>
+    </row>
+    <row r="559" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A559">
+        <v>2026007</v>
+      </c>
+      <c r="B559">
+        <v>2026</v>
+      </c>
+      <c r="C559" t="s">
+        <v>2695</v>
+      </c>
+      <c r="D559" t="s">
+        <v>2696</v>
+      </c>
+      <c r="E559" s="7" t="s">
+        <v>2693</v>
+      </c>
+      <c r="F559" t="s">
+        <v>2694</v>
+      </c>
+      <c r="G559" t="s">
+        <v>2689</v>
+      </c>
+      <c r="H559" t="s">
+        <v>2697</v>
+      </c>
+      <c r="I559" t="s">
+        <v>2299</v>
+      </c>
+      <c r="J559" t="s">
+        <v>2286</v>
+      </c>
+      <c r="K559" t="s">
+        <v>31</v>
+      </c>
+      <c r="L559" s="13" t="s">
+        <v>2691</v>
+      </c>
+      <c r="R559" s="8">
+        <v>64</v>
+      </c>
+      <c r="T559" s="4" t="s">
+        <v>2686</v>
+      </c>
+      <c r="V559">
+        <v>5</v>
+      </c>
+      <c r="W559" s="4" t="s">
+        <v>2383</v>
+      </c>
+      <c r="X559" t="s">
+        <v>2688</v>
+      </c>
+      <c r="Y559" t="s">
+        <v>2687</v>
+      </c>
+      <c r="Z559" t="s">
+        <v>2701</v>
+      </c>
+      <c r="AA559" t="s">
+        <v>2699</v>
+      </c>
+      <c r="AC559" s="1" t="s">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="560" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A560">
+        <v>2026007</v>
+      </c>
+      <c r="B560">
+        <v>2026</v>
+      </c>
+      <c r="C560" t="s">
+        <v>2695</v>
+      </c>
+      <c r="D560" t="s">
+        <v>2696</v>
+      </c>
+      <c r="E560" s="7" t="s">
+        <v>2693</v>
+      </c>
+      <c r="F560" t="s">
+        <v>2694</v>
+      </c>
+      <c r="G560" t="s">
+        <v>2690</v>
+      </c>
+      <c r="H560" t="s">
+        <v>2698</v>
+      </c>
+      <c r="I560" t="s">
+        <v>2299</v>
+      </c>
+      <c r="J560" t="s">
+        <v>2286</v>
+      </c>
+      <c r="K560" t="s">
+        <v>31</v>
+      </c>
+      <c r="L560" s="13" t="s">
+        <v>2692</v>
+      </c>
+      <c r="R560" s="8">
+        <v>120</v>
+      </c>
+      <c r="T560" s="4" t="s">
+        <v>2686</v>
+      </c>
+      <c r="V560">
+        <v>5</v>
+      </c>
+      <c r="W560" s="4" t="s">
+        <v>2383</v>
+      </c>
+      <c r="X560" t="s">
+        <v>2688</v>
+      </c>
+      <c r="Y560" t="s">
+        <v>2687</v>
+      </c>
+      <c r="Z560" t="s">
+        <v>2701</v>
+      </c>
+      <c r="AA560" t="s">
+        <v>2699</v>
+      </c>
+      <c r="AC560" s="1" t="s">
+        <v>2700</v>
       </c>
     </row>
   </sheetData>
@@ -45778,6 +46138,10 @@
     <hyperlink ref="AC123" r:id="rId482" xr:uid="{C3855FC3-DDDC-4C4A-842C-30A5DC0773F1}"/>
     <hyperlink ref="AC124" r:id="rId483" xr:uid="{39131C79-64A3-46F4-8781-29C747885AB7}"/>
     <hyperlink ref="AC125" r:id="rId484" xr:uid="{C621E5A7-94D6-49E5-ADCC-7CB2E6C065AE}"/>
+    <hyperlink ref="AC557" r:id="rId485" xr:uid="{1E54A5D6-0215-49AE-BA1C-80CEFCD22010}"/>
+    <hyperlink ref="AC558" r:id="rId486" xr:uid="{CF83D3C6-FB72-42D4-959C-86B6CA5968C7}"/>
+    <hyperlink ref="AC559" r:id="rId487" xr:uid="{4514D8B2-0385-474B-818B-2BDD94B50C43}"/>
+    <hyperlink ref="AC560" r:id="rId488" xr:uid="{B95077A5-B821-4945-A7B0-A42CC7202368}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>